<commit_message>
fix: ajusta alturas/anchos de columna, remueve Bitacora vacia, agrega cargo del responsable en 4 hojas
</commit_message>
<xml_diff>
--- a/backend/src/api/utils/template_inventario.xlsx
+++ b/backend/src/api/utils/template_inventario.xlsx
@@ -1845,7 +1845,7 @@
   <cols>
     <col width="4.5703125" customWidth="1" style="2" min="1" max="1"/>
     <col width="31.28515625" customWidth="1" min="2" max="2"/>
-    <col width="11.7109375" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="15" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="24.7109375" customWidth="1" min="4" max="4"/>
     <col width="11.28515625" bestFit="1" customWidth="1" min="5" max="5"/>
     <col width="8.140625" bestFit="1" customWidth="1" min="6" max="6"/>
@@ -2015,7 +2015,7 @@
     <row r="7" ht="15.75" customFormat="1" customHeight="1" s="5">
       <c r="B7" s="116" t="inlineStr">
         <is>
-          <t>CARGO DEL RESPONSABLE DE LA TOMA DEL INVENTARIO:</t>
+          <t>CARGO DEL RESPONSABLE DE LA TOMA DEL INVENTARIO: Profesional de servidores</t>
         </is>
       </c>
       <c r="C7" s="133" t="n"/>
@@ -2177,11 +2177,7 @@
           <t>Contrato Asociado</t>
         </is>
       </c>
-      <c r="T10" s="27" t="inlineStr">
-        <is>
-          <t>Bitacora</t>
-        </is>
-      </c>
+      <c r="T10" s="27" t="n"/>
       <c r="U10" s="28" t="n"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
@@ -18438,7 +18434,7 @@
     <row r="7" ht="15.95" customHeight="1" thickBot="1">
       <c r="B7" s="121" t="inlineStr">
         <is>
-          <t>CARGO DEL RESPONSABLE DE LA TOMA DEL INVENTARIO:</t>
+          <t>CARGO DEL RESPONSABLE DE LA TOMA DEL INVENTARIO: Profesional de redes</t>
         </is>
       </c>
       <c r="C7" s="142" t="n"/>
@@ -18549,11 +18545,7 @@
           <t>Contrato Asociado</t>
         </is>
       </c>
-      <c r="N10" s="31" t="inlineStr">
-        <is>
-          <t>Bitacora</t>
-        </is>
-      </c>
+      <c r="N10" s="31" t="n"/>
     </row>
     <row r="11" ht="30.75" customHeight="1">
       <c r="B11" s="32" t="inlineStr">
@@ -24423,9 +24415,9 @@
     <col width="22.85546875" customWidth="1" style="4" min="2" max="2"/>
     <col width="13.140625" customWidth="1" style="4" min="3" max="3"/>
     <col width="10.7109375" customWidth="1" style="4" min="4" max="4"/>
-    <col width="8.140625" customWidth="1" style="4" min="5" max="5"/>
+    <col width="14" customWidth="1" style="4" min="5" max="5"/>
     <col width="8.5703125" customWidth="1" style="4" min="6" max="6"/>
-    <col width="12.28515625" customWidth="1" style="4" min="7" max="7"/>
+    <col width="16" customWidth="1" style="4" min="7" max="7"/>
     <col width="10.140625" customWidth="1" style="4" min="8" max="8"/>
     <col width="13" customWidth="1" style="4" min="9" max="9"/>
     <col width="20.7109375" customWidth="1" style="4" min="10" max="10"/>
@@ -24522,7 +24514,7 @@
     <row r="7" ht="15.75" customFormat="1" customHeight="1" s="9">
       <c r="B7" s="121" t="inlineStr">
         <is>
-          <t>CARGO DEL RESPONSABLE DE LA TOMA DEL INVENTARIO:</t>
+          <t>CARGO DEL RESPONSABLE DE LA TOMA DEL INVENTARIO: Profesional de redes</t>
         </is>
       </c>
       <c r="C7" s="142" t="n"/>
@@ -24607,11 +24599,7 @@
           <t>Ubicación</t>
         </is>
       </c>
-      <c r="J10" s="125" t="inlineStr">
-        <is>
-          <t>Bitacora</t>
-        </is>
-      </c>
+      <c r="J10" s="125" t="n"/>
     </row>
     <row r="11" ht="30.75" customHeight="1">
       <c r="B11" s="35" t="inlineStr">
@@ -26561,7 +26549,7 @@
     <row r="7" ht="15.75" customHeight="1">
       <c r="B7" s="108" t="inlineStr">
         <is>
-          <t>CARGO DEL RESPONSABLE DE LA TOMA DEL INVENTARIO:</t>
+          <t>CARGO DEL RESPONSABLE DE LA TOMA DEL INVENTARIO: Administrador de base de datos</t>
         </is>
       </c>
       <c r="M7" s="136" t="n"/>
@@ -26652,11 +26640,7 @@
           <t>Contrato que lo soporta</t>
         </is>
       </c>
-      <c r="N10" s="72" t="inlineStr">
-        <is>
-          <t>Bitacora</t>
-        </is>
-      </c>
+      <c r="N10" s="72" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="73" t="inlineStr">

</xml_diff>